<commit_message>
Update Changelog, ExcelTemplates and Manual
</commit_message>
<xml_diff>
--- a/data/Excel/1.1.xlsx
+++ b/data/Excel/1.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\RAO_Project\data\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SHARE_3.95\Templates_win_only\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2163F1A6-8237-4529-8A9A-310B47E6EE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{908B8204-4775-4BD8-B3A9-01C62A207D40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.0" sheetId="3" r:id="rId1"/>
@@ -33,12 +33,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="73">
   <si>
     <t>Сведения об обособленном подразделении</t>
   </si>
@@ -80,42 +83,6 @@
   </si>
   <si>
     <t>Телефон</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Должность, фамилия, имя, отчество (при наличии) руководителя -                                                                                                   </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Адрес обособленного подразделения -                                                                                                     </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сокращенное наименование обособленного подразделения (при наличии) -                                                                                           </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Наименование обособленного подразделения -                                                                                                             </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Субъект Российской Федерации -                                                                                                                                                      </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Должность, фамилия, имя, отчество (при наличии) руководителя -       </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Адрес  места осуществления деятельности юридического лица -      </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Адрес юридического лица -          </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сокращенное наименование юридического лица (при наличии)-   </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Наименование юридического лица -    </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Субъект Российской Федерации - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Орган управления использованием атомной энергии -                                                                                                                                        </t>
   </si>
   <si>
     <t>2. Воинские части (организации) Вооруженных Сил Российской Федерации:
@@ -301,6 +268,36 @@
   </si>
   <si>
     <t>Дата окончания настоящего отчетного периода</t>
+  </si>
+  <si>
+    <t>Орган управления использованием атомной энергии</t>
+  </si>
+  <si>
+    <t>Субъект Российской Федерации</t>
+  </si>
+  <si>
+    <t>Наименование юридического лица</t>
+  </si>
+  <si>
+    <t>Сокращенное наименование юридического лица (при наличии)</t>
+  </si>
+  <si>
+    <t>Адрес юридического лица</t>
+  </si>
+  <si>
+    <t>Адрес  места осуществления деятельности юридического лица</t>
+  </si>
+  <si>
+    <t>Должность, фамилия, имя, отчество (при наличии) руководителя</t>
+  </si>
+  <si>
+    <t>Наименование обособленного подразделения</t>
+  </si>
+  <si>
+    <t>Адрес обособленного подразделения</t>
+  </si>
+  <si>
+    <t>Сокращенное наименование обособленного подразделения (при наличии)</t>
   </si>
 </sst>
 </file>
@@ -491,19 +488,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -841,6 +825,19 @@
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -850,7 +847,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -863,12 +860,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -898,74 +889,114 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -976,106 +1007,85 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -1087,23 +1097,28 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="4"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="4"/>
@@ -1123,32 +1138,38 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1436,387 +1457,387 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I37"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.7265625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.81640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.453125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.81640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="40.26953125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="37.453125" style="1" customWidth="1"/>
-    <col min="7" max="9" width="10.54296875" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.1796875" style="1"/>
+    <col min="1" max="1" width="16.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="40.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="37.42578125" style="1" customWidth="1"/>
+    <col min="7" max="9" width="10.5703125" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="I1" s="12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="79" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="80" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" s="80"/>
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="80"/>
-    </row>
-    <row r="4" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="80" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="80"/>
-      <c r="C4" s="80"/>
-      <c r="D4" s="80"/>
-      <c r="E4" s="80"/>
-      <c r="F4" s="80"/>
-      <c r="G4" s="80"/>
-      <c r="H4" s="80"/>
-      <c r="I4" s="80"/>
-    </row>
-    <row r="5" spans="1:9" ht="2.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="27"/>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-    </row>
-    <row r="6" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D6" s="11"/>
-      <c r="E6" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="30"/>
-      <c r="G6" s="10" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="76" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" s="77"/>
-      <c r="C10" s="77"/>
-      <c r="D10" s="77"/>
-      <c r="E10" s="78"/>
-      <c r="F10" s="75" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="86.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="69" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="70"/>
-      <c r="C11" s="70"/>
-      <c r="D11" s="70"/>
-      <c r="E11" s="71"/>
-      <c r="F11" s="75"/>
-    </row>
-    <row r="12" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="69" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="70"/>
-      <c r="C12" s="70"/>
-      <c r="D12" s="70"/>
-      <c r="E12" s="71"/>
-      <c r="F12" s="75"/>
-    </row>
-    <row r="13" spans="1:9" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="69"/>
-      <c r="B13" s="70"/>
-      <c r="C13" s="70"/>
-      <c r="D13" s="70"/>
-      <c r="E13" s="71"/>
-      <c r="F13" s="75"/>
-    </row>
-    <row r="14" spans="1:9" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="72"/>
-      <c r="B14" s="73"/>
-      <c r="C14" s="73"/>
-      <c r="D14" s="73"/>
-      <c r="E14" s="74"/>
-      <c r="F14" s="75"/>
-    </row>
-    <row r="15" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="63" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="64"/>
-      <c r="C15" s="64"/>
-      <c r="D15" s="64"/>
-      <c r="E15" s="65"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="41"/>
-    </row>
-    <row r="16" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="48" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I1" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="74" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
+      <c r="I2" s="74"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="75" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="75"/>
+      <c r="C3" s="75"/>
+      <c r="D3" s="75"/>
+      <c r="E3" s="75"/>
+      <c r="F3" s="75"/>
+      <c r="G3" s="75"/>
+      <c r="H3" s="75"/>
+      <c r="I3" s="75"/>
+    </row>
+    <row r="4" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="75" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="75"/>
+      <c r="C4" s="75"/>
+      <c r="D4" s="75"/>
+      <c r="E4" s="75"/>
+      <c r="F4" s="75"/>
+      <c r="G4" s="75"/>
+      <c r="H4" s="75"/>
+      <c r="I4" s="75"/>
+    </row>
+    <row r="5" spans="1:9" ht="2.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="21"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+    </row>
+    <row r="6" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D6" s="9"/>
+      <c r="E6" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="23"/>
+      <c r="G6" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="71" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="72"/>
+      <c r="C10" s="72"/>
+      <c r="D10" s="72"/>
+      <c r="E10" s="73"/>
+      <c r="F10" s="70" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="86.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="64" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="65"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="65"/>
+      <c r="E11" s="66"/>
+      <c r="F11" s="70"/>
+    </row>
+    <row r="12" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="64" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="65"/>
+      <c r="C12" s="65"/>
+      <c r="D12" s="65"/>
+      <c r="E12" s="66"/>
+      <c r="F12" s="70"/>
+    </row>
+    <row r="13" spans="1:9" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="64"/>
+      <c r="B13" s="65"/>
+      <c r="C13" s="65"/>
+      <c r="D13" s="65"/>
+      <c r="E13" s="66"/>
+      <c r="F13" s="70"/>
+    </row>
+    <row r="14" spans="1:9" ht="30.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="67"/>
+      <c r="B14" s="68"/>
+      <c r="C14" s="68"/>
+      <c r="D14" s="68"/>
+      <c r="E14" s="69"/>
+      <c r="F14" s="70"/>
+    </row>
+    <row r="15" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="61" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="61"/>
+      <c r="C15" s="61"/>
+      <c r="D15" s="61"/>
+      <c r="E15" s="61"/>
+      <c r="F15" s="43"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="45"/>
+    </row>
+    <row r="16" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B16" s="67" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="67"/>
-      <c r="D16" s="67"/>
-      <c r="E16" s="68"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="34"/>
-      <c r="I16" s="35"/>
-    </row>
-    <row r="17" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="48"/>
+      <c r="B16" s="63" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="63"/>
+      <c r="D16" s="63"/>
+      <c r="E16" s="63"/>
+      <c r="F16" s="37"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="39"/>
+    </row>
+    <row r="17" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="62"/>
       <c r="B17" s="52" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="C17" s="52"/>
       <c r="D17" s="52"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="34"/>
-      <c r="I17" s="35"/>
-    </row>
-    <row r="18" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="48"/>
+      <c r="E17" s="52"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="39"/>
+    </row>
+    <row r="18" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="62"/>
       <c r="B18" s="52" t="s">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="C18" s="52"/>
       <c r="D18" s="52"/>
-      <c r="E18" s="53"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="34"/>
-      <c r="I18" s="35"/>
-    </row>
-    <row r="19" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="48"/>
+      <c r="E18" s="52"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="38"/>
+      <c r="H18" s="38"/>
+      <c r="I18" s="39"/>
+    </row>
+    <row r="19" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="62"/>
       <c r="B19" s="52" t="s">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="C19" s="52"/>
       <c r="D19" s="52"/>
-      <c r="E19" s="53"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="34"/>
-      <c r="I19" s="35"/>
-    </row>
-    <row r="20" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="48"/>
+      <c r="E19" s="52"/>
+      <c r="F19" s="37"/>
+      <c r="G19" s="38"/>
+      <c r="H19" s="38"/>
+      <c r="I19" s="39"/>
+    </row>
+    <row r="20" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="62"/>
       <c r="B20" s="52" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C20" s="52"/>
       <c r="D20" s="52"/>
-      <c r="E20" s="53"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="34"/>
-      <c r="I20" s="35"/>
-    </row>
-    <row r="21" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="48"/>
+      <c r="E20" s="52"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="38"/>
+      <c r="H20" s="38"/>
+      <c r="I20" s="39"/>
+    </row>
+    <row r="21" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="62"/>
       <c r="B21" s="52" t="s">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="C21" s="52"/>
       <c r="D21" s="52"/>
-      <c r="E21" s="53"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="35"/>
-    </row>
-    <row r="22" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="48"/>
-      <c r="B22" s="54" t="s">
+      <c r="E21" s="52"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="38"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="39"/>
+    </row>
+    <row r="22" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="62"/>
+      <c r="B22" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="54"/>
-      <c r="D22" s="54"/>
-      <c r="E22" s="55"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="34"/>
-      <c r="I22" s="35"/>
-    </row>
-    <row r="23" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="48"/>
-      <c r="B23" s="54" t="s">
+      <c r="C22" s="53"/>
+      <c r="D22" s="53"/>
+      <c r="E22" s="53"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="38"/>
+      <c r="I22" s="39"/>
+    </row>
+    <row r="23" spans="1:9" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="62"/>
+      <c r="B23" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="C23" s="54"/>
-      <c r="D23" s="54"/>
-      <c r="E23" s="55"/>
-      <c r="F23" s="33"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="35"/>
-    </row>
-    <row r="24" spans="1:9" ht="23.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="66"/>
-      <c r="B24" s="45" t="s">
+      <c r="C23" s="53"/>
+      <c r="D23" s="53"/>
+      <c r="E23" s="53"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="38"/>
+      <c r="I23" s="39"/>
+    </row>
+    <row r="24" spans="1:9" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="62"/>
+      <c r="B24" s="49" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="45"/>
-      <c r="D24" s="45"/>
-      <c r="E24" s="46"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="37"/>
-      <c r="I24" s="38"/>
-    </row>
-    <row r="25" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="47" t="s">
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="41"/>
+      <c r="H24" s="41"/>
+      <c r="I24" s="42"/>
+    </row>
+    <row r="25" spans="1:9" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="B25" s="50" t="s">
-        <v>18</v>
-      </c>
-      <c r="C25" s="50"/>
-      <c r="D25" s="50"/>
+      <c r="B25" s="51" t="s">
+        <v>64</v>
+      </c>
+      <c r="C25" s="51"/>
+      <c r="D25" s="51"/>
       <c r="E25" s="51"/>
-      <c r="F25" s="58"/>
-      <c r="G25" s="59"/>
-      <c r="H25" s="59"/>
-      <c r="I25" s="60"/>
-    </row>
-    <row r="26" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="48"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="56"/>
+      <c r="H25" s="56"/>
+      <c r="I25" s="57"/>
+    </row>
+    <row r="26" spans="1:9" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="50"/>
       <c r="B26" s="52" t="s">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="C26" s="52"/>
       <c r="D26" s="52"/>
-      <c r="E26" s="53"/>
-      <c r="F26" s="61"/>
-      <c r="G26" s="52"/>
-      <c r="H26" s="52"/>
-      <c r="I26" s="62"/>
-    </row>
-    <row r="27" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="48"/>
+      <c r="E26" s="52"/>
+      <c r="F26" s="58"/>
+      <c r="G26" s="59"/>
+      <c r="H26" s="59"/>
+      <c r="I26" s="60"/>
+    </row>
+    <row r="27" spans="1:9" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="50"/>
       <c r="B27" s="52" t="s">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="C27" s="52"/>
       <c r="D27" s="52"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="61"/>
-      <c r="G27" s="52"/>
-      <c r="H27" s="52"/>
-      <c r="I27" s="62"/>
-    </row>
-    <row r="28" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="48"/>
+      <c r="E27" s="52"/>
+      <c r="F27" s="58"/>
+      <c r="G27" s="59"/>
+      <c r="H27" s="59"/>
+      <c r="I27" s="60"/>
+    </row>
+    <row r="28" spans="1:9" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="50"/>
       <c r="B28" s="52" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="C28" s="52"/>
       <c r="D28" s="52"/>
-      <c r="E28" s="53"/>
-      <c r="F28" s="61"/>
-      <c r="G28" s="52"/>
-      <c r="H28" s="52"/>
-      <c r="I28" s="62"/>
-    </row>
-    <row r="29" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="48"/>
+      <c r="E28" s="52"/>
+      <c r="F28" s="58"/>
+      <c r="G28" s="59"/>
+      <c r="H28" s="59"/>
+      <c r="I28" s="60"/>
+    </row>
+    <row r="29" spans="1:9" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="50"/>
       <c r="B29" s="52" t="s">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="C29" s="52"/>
       <c r="D29" s="52"/>
-      <c r="E29" s="53"/>
-      <c r="F29" s="61"/>
-      <c r="G29" s="52"/>
-      <c r="H29" s="52"/>
-      <c r="I29" s="62"/>
-    </row>
-    <row r="30" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="48"/>
-      <c r="B30" s="54" t="s">
+      <c r="E29" s="52"/>
+      <c r="F29" s="58"/>
+      <c r="G29" s="59"/>
+      <c r="H29" s="59"/>
+      <c r="I29" s="60"/>
+    </row>
+    <row r="30" spans="1:9" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="50"/>
+      <c r="B30" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="C30" s="54"/>
-      <c r="D30" s="54"/>
-      <c r="E30" s="55"/>
-      <c r="F30" s="33"/>
-      <c r="G30" s="34"/>
-      <c r="H30" s="34"/>
-      <c r="I30" s="35"/>
-    </row>
-    <row r="31" spans="1:9" ht="23.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="48"/>
-      <c r="B31" s="54" t="s">
+      <c r="C30" s="53"/>
+      <c r="D30" s="53"/>
+      <c r="E30" s="53"/>
+      <c r="F30" s="37"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="39"/>
+    </row>
+    <row r="31" spans="1:9" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="50"/>
+      <c r="B31" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="C31" s="54"/>
-      <c r="D31" s="54"/>
-      <c r="E31" s="55"/>
-      <c r="F31" s="33"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="35"/>
-    </row>
-    <row r="32" spans="1:9" ht="23.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="49"/>
-      <c r="B32" s="56" t="s">
+      <c r="C31" s="53"/>
+      <c r="D31" s="53"/>
+      <c r="E31" s="53"/>
+      <c r="F31" s="37"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="39"/>
+    </row>
+    <row r="32" spans="1:9" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="50"/>
+      <c r="B32" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="C32" s="56"/>
-      <c r="D32" s="56"/>
-      <c r="E32" s="57"/>
-      <c r="F32" s="36"/>
-      <c r="G32" s="37"/>
-      <c r="H32" s="37"/>
-      <c r="I32" s="38"/>
-    </row>
-    <row r="33" spans="1:9" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="G33" s="9"/>
-    </row>
-    <row r="34" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="42" t="s">
+      <c r="C32" s="54"/>
+      <c r="D32" s="54"/>
+      <c r="E32" s="54"/>
+      <c r="F32" s="40"/>
+      <c r="G32" s="41"/>
+      <c r="H32" s="41"/>
+      <c r="I32" s="42"/>
+    </row>
+    <row r="33" spans="1:9" ht="23.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G33" s="7"/>
+    </row>
+    <row r="34" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="B34" s="43"/>
-      <c r="C34" s="43"/>
-      <c r="D34" s="43"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="43"/>
-      <c r="I34" s="44"/>
-    </row>
-    <row r="35" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B34" s="47"/>
+      <c r="C34" s="47"/>
+      <c r="D34" s="47"/>
+      <c r="E34" s="47"/>
+      <c r="F34" s="47"/>
+      <c r="G34" s="47"/>
+      <c r="H34" s="47"/>
+      <c r="I34" s="48"/>
+    </row>
+    <row r="35" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4"/>
       <c r="B35" s="3" t="s">
         <v>9</v>
@@ -1843,33 +1864,34 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:9" s="2" customFormat="1" ht="47" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="8" t="s">
+    <row r="36" spans="1:9" s="2" customFormat="1" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B36" s="7"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-    </row>
-    <row r="37" spans="1:9" s="2" customFormat="1" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B36" s="24"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="25"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="25"/>
+      <c r="I36" s="25"/>
+    </row>
+    <row r="37" spans="1:9" s="2" customFormat="1" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B37" s="4"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
-      <c r="I37" s="3"/>
+      <c r="B37" s="26"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="27"/>
+      <c r="H37" s="27"/>
+      <c r="I37" s="27"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="UVPpGGZOFPKR1EAkJ7VgGrTG0NZyKQWm0/1j97NIi7J5MrMPAIH/w0NDehWVBQ/6j8agrGrCemrDrETJbXALeA==" saltValue="P3io2/U7X6YfHSbTfxE/IQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0"/>
   <mergeCells count="46">
     <mergeCell ref="A12:E14"/>
     <mergeCell ref="F10:F14"/>
@@ -1929,459 +1951,467 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:W19"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="5" width="10.54296875" style="13" customWidth="1"/>
-    <col min="6" max="23" width="10.54296875" style="14" customWidth="1"/>
-    <col min="24" max="16384" width="8.81640625" style="14"/>
+    <col min="1" max="5" width="10.5703125" style="11" customWidth="1"/>
+    <col min="6" max="23" width="10.5703125" style="12" customWidth="1"/>
+    <col min="24" max="16384" width="8.85546875" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="W1" s="15" t="s">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="W1" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="85" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="86"/>
+      <c r="C2" s="86"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
+      <c r="H2" s="86"/>
+      <c r="I2" s="86"/>
+      <c r="J2" s="86"/>
+      <c r="K2" s="86"/>
+      <c r="L2" s="86"/>
+      <c r="M2" s="86"/>
+      <c r="N2" s="86"/>
+      <c r="O2" s="86"/>
+      <c r="P2" s="86"/>
+      <c r="Q2" s="86"/>
+      <c r="R2" s="86"/>
+      <c r="S2" s="86"/>
+      <c r="T2" s="86"/>
+      <c r="U2" s="86"/>
+      <c r="V2" s="86"/>
+      <c r="W2" s="86"/>
+    </row>
+    <row r="3" spans="1:23" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="87" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="87"/>
+      <c r="C3" s="87"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="96"/>
+      <c r="H3" s="96"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
+      <c r="O3" s="14"/>
+      <c r="P3" s="14"/>
+      <c r="Q3" s="14"/>
+      <c r="R3" s="14"/>
+      <c r="S3" s="14"/>
+      <c r="T3" s="14"/>
+      <c r="U3" s="14"/>
+      <c r="V3" s="14"/>
+      <c r="W3" s="14"/>
+    </row>
+    <row r="4" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="87" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="87"/>
+      <c r="C4" s="87"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="87"/>
+      <c r="F4" s="87"/>
+      <c r="G4" s="97"/>
+      <c r="H4" s="97"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="14"/>
+      <c r="P4" s="14"/>
+      <c r="Q4" s="14"/>
+      <c r="R4" s="14"/>
+      <c r="S4" s="14"/>
+      <c r="T4" s="14"/>
+      <c r="U4" s="14"/>
+      <c r="V4" s="14"/>
+      <c r="W4" s="14"/>
+    </row>
+    <row r="5" spans="1:23" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="87" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="87"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="87"/>
+      <c r="F5" s="87"/>
+      <c r="G5" s="98"/>
+      <c r="H5" s="98"/>
+    </row>
+    <row r="6" spans="1:23" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="15"/>
+    </row>
+    <row r="7" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="88" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="90" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="91"/>
+      <c r="D7" s="90" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="94"/>
+      <c r="F7" s="94"/>
+      <c r="G7" s="94"/>
+      <c r="H7" s="94"/>
+      <c r="I7" s="94"/>
+      <c r="J7" s="94"/>
+      <c r="K7" s="94"/>
+      <c r="L7" s="94"/>
+      <c r="M7" s="91"/>
+      <c r="N7" s="90" t="s">
+        <v>61</v>
+      </c>
+      <c r="O7" s="91"/>
+      <c r="P7" s="90" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q7" s="94"/>
+      <c r="R7" s="91"/>
+      <c r="S7" s="90" t="s">
+        <v>32</v>
+      </c>
+      <c r="T7" s="91"/>
+      <c r="U7" s="90" t="s">
+        <v>33</v>
+      </c>
+      <c r="V7" s="94"/>
+      <c r="W7" s="91"/>
+    </row>
+    <row r="8" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="89"/>
+      <c r="B8" s="92"/>
+      <c r="C8" s="93"/>
+      <c r="D8" s="92"/>
+      <c r="E8" s="95"/>
+      <c r="F8" s="95"/>
+      <c r="G8" s="95"/>
+      <c r="H8" s="95"/>
+      <c r="I8" s="95"/>
+      <c r="J8" s="95"/>
+      <c r="K8" s="95"/>
+      <c r="L8" s="95"/>
+      <c r="M8" s="93"/>
+      <c r="N8" s="92"/>
+      <c r="O8" s="93"/>
+      <c r="P8" s="92"/>
+      <c r="Q8" s="95"/>
+      <c r="R8" s="93"/>
+      <c r="S8" s="92"/>
+      <c r="T8" s="93"/>
+      <c r="U8" s="92"/>
+      <c r="V8" s="95"/>
+      <c r="W8" s="93"/>
+    </row>
+    <row r="9" spans="1:23" ht="320.10000000000002" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="89"/>
+      <c r="B9" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="18" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="2" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="90" t="s">
+      <c r="E9" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="91"/>
-      <c r="C2" s="91"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
-      <c r="H2" s="91"/>
-      <c r="I2" s="91"/>
-      <c r="J2" s="91"/>
-      <c r="K2" s="91"/>
-      <c r="L2" s="91"/>
-      <c r="M2" s="91"/>
-      <c r="N2" s="91"/>
-      <c r="O2" s="91"/>
-      <c r="P2" s="91"/>
-      <c r="Q2" s="91"/>
-      <c r="R2" s="91"/>
-      <c r="S2" s="91"/>
-      <c r="T2" s="91"/>
-      <c r="U2" s="91"/>
-      <c r="V2" s="91"/>
-      <c r="W2" s="91"/>
-    </row>
-    <row r="3" spans="1:23" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="92" t="s">
+      <c r="F9" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="92"/>
-      <c r="C3" s="92"/>
-      <c r="D3" s="92"/>
-      <c r="E3" s="92"/>
-      <c r="F3" s="92"/>
-      <c r="G3" s="100"/>
-      <c r="H3" s="100"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
-      <c r="N3" s="16"/>
-      <c r="O3" s="16"/>
-      <c r="P3" s="16"/>
-      <c r="Q3" s="16"/>
-      <c r="R3" s="16"/>
-      <c r="S3" s="16"/>
-      <c r="T3" s="16"/>
-      <c r="U3" s="16"/>
-      <c r="V3" s="16"/>
-      <c r="W3" s="16"/>
-    </row>
-    <row r="4" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="92" t="s">
-        <v>74</v>
-      </c>
-      <c r="B4" s="92"/>
-      <c r="C4" s="92"/>
-      <c r="D4" s="92"/>
-      <c r="E4" s="92"/>
-      <c r="F4" s="92"/>
-      <c r="G4" s="101"/>
-      <c r="H4" s="101"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16"/>
-      <c r="N4" s="16"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="16"/>
-      <c r="Q4" s="16"/>
-      <c r="R4" s="16"/>
-      <c r="S4" s="16"/>
-      <c r="T4" s="16"/>
-      <c r="U4" s="16"/>
-      <c r="V4" s="16"/>
-      <c r="W4" s="16"/>
-    </row>
-    <row r="5" spans="1:23" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="92" t="s">
+      <c r="G9" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="92"/>
-      <c r="C5" s="92"/>
-      <c r="D5" s="92"/>
-      <c r="E5" s="92"/>
-      <c r="F5" s="92"/>
-      <c r="G5" s="102"/>
-      <c r="H5" s="102"/>
-    </row>
-    <row r="6" spans="1:23" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="18"/>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="17"/>
-    </row>
-    <row r="7" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="93" t="s">
+      <c r="H9" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="95" t="s">
+      <c r="I9" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="96"/>
-      <c r="D7" s="95" t="s">
+      <c r="J9" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="99"/>
-      <c r="F7" s="99"/>
-      <c r="G7" s="99"/>
-      <c r="H7" s="99"/>
-      <c r="I7" s="99"/>
-      <c r="J7" s="99"/>
-      <c r="K7" s="99"/>
-      <c r="L7" s="99"/>
-      <c r="M7" s="96"/>
-      <c r="N7" s="95" t="s">
-        <v>73</v>
-      </c>
-      <c r="O7" s="96"/>
-      <c r="P7" s="95" t="s">
+      <c r="K9" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="Q7" s="99"/>
-      <c r="R7" s="96"/>
-      <c r="S7" s="95" t="s">
+      <c r="L9" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="T7" s="96"/>
-      <c r="U7" s="95" t="s">
+      <c r="M9" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="V7" s="99"/>
-      <c r="W7" s="96"/>
-    </row>
-    <row r="8" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="94"/>
-      <c r="B8" s="97"/>
-      <c r="C8" s="98"/>
-      <c r="D8" s="97"/>
-      <c r="E8" s="82"/>
-      <c r="F8" s="82"/>
-      <c r="G8" s="82"/>
-      <c r="H8" s="82"/>
-      <c r="I8" s="82"/>
-      <c r="J8" s="82"/>
-      <c r="K8" s="82"/>
-      <c r="L8" s="82"/>
-      <c r="M8" s="98"/>
-      <c r="N8" s="97"/>
-      <c r="O8" s="98"/>
-      <c r="P8" s="97"/>
-      <c r="Q8" s="82"/>
-      <c r="R8" s="98"/>
-      <c r="S8" s="97"/>
-      <c r="T8" s="98"/>
-      <c r="U8" s="97"/>
-      <c r="V8" s="82"/>
-      <c r="W8" s="98"/>
-    </row>
-    <row r="9" spans="1:23" ht="320.14999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="94"/>
-      <c r="B9" s="19" t="s">
+      <c r="N9" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="O9" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="P9" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="E9" s="20" t="s">
+      <c r="Q9" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="R9" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="S9" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="T9" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="U9" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="H9" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="I9" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="J9" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="K9" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="L9" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="M9" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="N9" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="O9" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="P9" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q9" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="R9" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="S9" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="T9" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="U9" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="V9" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="W9" s="20" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="V9" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="W9" s="18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" s="30" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="28">
         <v>1</v>
       </c>
-      <c r="B10" s="22">
+      <c r="B10" s="29">
         <v>2</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="29">
         <v>3</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="29">
         <v>4</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="29">
         <v>5</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="29">
         <v>6</v>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="29">
         <v>7</v>
       </c>
-      <c r="H10" s="22">
+      <c r="H10" s="29">
         <v>8</v>
       </c>
-      <c r="I10" s="22">
+      <c r="I10" s="29">
         <v>9</v>
       </c>
-      <c r="J10" s="22">
+      <c r="J10" s="29">
         <v>10</v>
       </c>
-      <c r="K10" s="22">
+      <c r="K10" s="29">
         <v>11</v>
       </c>
-      <c r="L10" s="22">
+      <c r="L10" s="29">
         <v>12</v>
       </c>
-      <c r="M10" s="22">
+      <c r="M10" s="29">
         <v>13</v>
       </c>
-      <c r="N10" s="22">
+      <c r="N10" s="29">
         <v>14</v>
       </c>
-      <c r="O10" s="22">
+      <c r="O10" s="29">
         <v>15</v>
       </c>
-      <c r="P10" s="22">
+      <c r="P10" s="29">
         <v>16</v>
       </c>
-      <c r="Q10" s="22">
+      <c r="Q10" s="29">
         <v>17</v>
       </c>
-      <c r="R10" s="22">
+      <c r="R10" s="29">
         <v>18</v>
       </c>
-      <c r="S10" s="22">
+      <c r="S10" s="29">
         <v>19</v>
       </c>
-      <c r="T10" s="22">
+      <c r="T10" s="29">
         <v>20</v>
       </c>
-      <c r="U10" s="22">
+      <c r="U10" s="29">
         <v>21</v>
       </c>
-      <c r="V10" s="22">
+      <c r="V10" s="29">
         <v>22</v>
       </c>
-      <c r="W10" s="22">
+      <c r="W10" s="29">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="15.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="21"/>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="21"/>
-      <c r="L11" s="21"/>
-      <c r="M11" s="21"/>
-      <c r="N11" s="21"/>
-      <c r="O11" s="21"/>
-      <c r="P11" s="21"/>
-      <c r="Q11" s="21"/>
-      <c r="R11" s="21"/>
-      <c r="S11" s="21"/>
-      <c r="T11" s="21"/>
-      <c r="U11" s="21"/>
-      <c r="V11" s="21"/>
-      <c r="W11" s="21"/>
-    </row>
-    <row r="13" spans="1:23" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-    </row>
-    <row r="14" spans="1:23" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="32" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="C14" s="84" t="s">
-        <v>67</v>
-      </c>
-      <c r="D14" s="85"/>
-      <c r="E14" s="85"/>
-      <c r="F14" s="85"/>
-      <c r="G14" s="85"/>
-      <c r="H14" s="85"/>
-      <c r="I14" s="85"/>
-      <c r="J14" s="85"/>
-      <c r="K14" s="85"/>
-      <c r="L14" s="86"/>
-    </row>
-    <row r="15" spans="1:23" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="32"/>
-      <c r="B15" s="31"/>
-      <c r="C15" s="84"/>
-      <c r="D15" s="85"/>
-      <c r="E15" s="85"/>
-      <c r="F15" s="85"/>
-      <c r="G15" s="85"/>
-      <c r="H15" s="85"/>
-      <c r="I15" s="85"/>
-      <c r="J15" s="85"/>
-      <c r="K15" s="85"/>
-      <c r="L15" s="86"/>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A16" s="23"/>
-      <c r="B16" s="87"/>
-      <c r="C16" s="87"/>
-      <c r="D16" s="87"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A17" s="24"/>
-      <c r="B17" s="88"/>
-      <c r="C17" s="88"/>
-      <c r="D17" s="88"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="24"/>
-      <c r="I17" s="24"/>
-      <c r="J17" s="24"/>
-      <c r="K17" s="24"/>
-      <c r="L17" s="24"/>
-    </row>
-    <row r="18" spans="1:12" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="89" t="s">
-        <v>68</v>
-      </c>
-      <c r="B18" s="89"/>
-      <c r="C18" s="89"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="82"/>
-      <c r="G18" s="82"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="25"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="82"/>
-      <c r="L18" s="82"/>
-    </row>
-    <row r="19" spans="1:12" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="24"/>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="E19" s="29"/>
-      <c r="F19" s="81" t="s">
-        <v>70</v>
-      </c>
-      <c r="G19" s="81"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26" t="s">
-        <v>71</v>
-      </c>
-      <c r="J19" s="26"/>
-      <c r="K19" s="83" t="s">
-        <v>72</v>
-      </c>
-      <c r="L19" s="83"/>
+    <row r="11" spans="1:23" s="30" customFormat="1" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="31"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="31"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="31"/>
+      <c r="L11" s="31"/>
+      <c r="M11" s="31"/>
+      <c r="N11" s="31"/>
+      <c r="O11" s="31"/>
+      <c r="P11" s="31"/>
+      <c r="Q11" s="31"/>
+      <c r="R11" s="31"/>
+      <c r="S11" s="31"/>
+      <c r="T11" s="31"/>
+      <c r="U11" s="31"/>
+      <c r="V11" s="31"/>
+      <c r="W11" s="31"/>
+    </row>
+    <row r="12" spans="1:23" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="32"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+    </row>
+    <row r="13" spans="1:23" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+    </row>
+    <row r="14" spans="1:23" s="30" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="79" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="80"/>
+      <c r="E14" s="80"/>
+      <c r="F14" s="80"/>
+      <c r="G14" s="80"/>
+      <c r="H14" s="80"/>
+      <c r="I14" s="80"/>
+      <c r="J14" s="80"/>
+      <c r="K14" s="80"/>
+      <c r="L14" s="81"/>
+    </row>
+    <row r="15" spans="1:23" s="30" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="33"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="79"/>
+      <c r="D15" s="80"/>
+      <c r="E15" s="80"/>
+      <c r="F15" s="80"/>
+      <c r="G15" s="80"/>
+      <c r="H15" s="80"/>
+      <c r="I15" s="80"/>
+      <c r="J15" s="80"/>
+      <c r="K15" s="80"/>
+      <c r="L15" s="81"/>
+    </row>
+    <row r="16" spans="1:23" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="35"/>
+      <c r="B16" s="82"/>
+      <c r="C16" s="82"/>
+      <c r="D16" s="82"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="35"/>
+      <c r="G16" s="35"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="35"/>
+      <c r="J16" s="35"/>
+      <c r="K16" s="35"/>
+      <c r="L16" s="35"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="19"/>
+      <c r="B17" s="83"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="83"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="19"/>
+      <c r="K17" s="19"/>
+      <c r="L17" s="19"/>
+    </row>
+    <row r="18" spans="1:12" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="84" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="84"/>
+      <c r="C18" s="84"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="77"/>
+      <c r="G18" s="77"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="36"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="77"/>
+      <c r="L18" s="77"/>
+    </row>
+    <row r="19" spans="1:12" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="19"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="E19" s="22"/>
+      <c r="F19" s="76" t="s">
+        <v>58</v>
+      </c>
+      <c r="G19" s="76"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="J19" s="20"/>
+      <c r="K19" s="78" t="s">
+        <v>60</v>
+      </c>
+      <c r="L19" s="78"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="JwNw2mwtYT9IM1wu7OXaASZVQ1Zu0JrEu2DAvj8yT7nV2l5PC9u90TD7UDL376V7jT3x4oj3M9w0YgvWJkkygQ==" saltValue="/X1UWRa4l3plVY3H9xA3eQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" insertRows="0"/>
   <mergeCells count="23">
     <mergeCell ref="A2:W2"/>
     <mergeCell ref="A3:F3"/>

</xml_diff>